<commit_message>
Update final correlation matrix for full seven-model sample
</commit_message>
<xml_diff>
--- a/src/econometrics/wp07_reestimation/Final_spec_correlation_matrix.xlsx
+++ b/src/econometrics/wp07_reestimation/Final_spec_correlation_matrix.xlsx
@@ -2271,7 +2271,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>3918</v>
+        <v>4648</v>
       </c>
     </row>
     <row r="4">
@@ -2318,34 +2318,34 @@
         <v>1</v>
       </c>
       <c r="C5" s="15">
-        <v>0.023100696701153303</v>
+        <v>0.033988950952882471</v>
       </c>
       <c r="D5" s="16">
-        <v>-0.17855825511226522</v>
+        <v>-0.13993747861363737</v>
       </c>
       <c r="E5" s="17">
-        <v>-0.13252929003989472</v>
+        <v>-0.072168942664718683</v>
       </c>
       <c r="F5" s="18">
-        <v>-0.16158769856153238</v>
+        <v>-0.16020229891420215</v>
       </c>
       <c r="G5" s="19">
-        <v>-0.078605187138131694</v>
+        <v>-0.036455441011521955</v>
       </c>
       <c r="H5" s="20">
-        <v>0.0039272163451361287</v>
+        <v>0.051208472342005616</v>
       </c>
       <c r="I5" s="21">
-        <v>-0.18790273986482514</v>
+        <v>-0.16107412495124424</v>
       </c>
       <c r="J5" s="22">
-        <v>-0.086944371736145623</v>
+        <v>-0.074643708637271544</v>
       </c>
       <c r="K5" s="23">
-        <v>-0.053100175798924773</v>
+        <v>-0.053667623229320345</v>
       </c>
       <c r="L5" s="24">
-        <v>-0.31364711226513603</v>
+        <v>-0.30695290477763448</v>
       </c>
     </row>
     <row r="6">
@@ -2353,37 +2353,37 @@
         <v>3</v>
       </c>
       <c r="B6" s="26">
-        <v>0.023100696701153303</v>
+        <v>0.033988950952882471</v>
       </c>
       <c r="C6" s="27">
         <v>1</v>
       </c>
       <c r="D6" s="28">
-        <v>-0.35685101244146372</v>
+        <v>-0.27945448217603419</v>
       </c>
       <c r="E6" s="29">
-        <v>0.45723953115542315</v>
+        <v>0.3912405587965328</v>
       </c>
       <c r="F6" s="30">
-        <v>-0.19866141481895314</v>
+        <v>-0.16779261703691015</v>
       </c>
       <c r="G6" s="31">
-        <v>-0.11068638947112709</v>
+        <v>-0.082947729960389002</v>
       </c>
       <c r="H6" s="32">
-        <v>0.35783377533033073</v>
+        <v>0.25181928605750192</v>
       </c>
       <c r="I6" s="33">
-        <v>0.18904785927448819</v>
+        <v>0.13795657281457507</v>
       </c>
       <c r="J6" s="34">
-        <v>0.0082009235447547887</v>
+        <v>0.0034549274764648146</v>
       </c>
       <c r="K6" s="35">
-        <v>-0.0032735505005431517</v>
+        <v>-0.0051518167771299923</v>
       </c>
       <c r="L6" s="36">
-        <v>-0.038354854119573539</v>
+        <v>-0.037623278440063204</v>
       </c>
     </row>
     <row r="7">
@@ -2391,37 +2391,37 @@
         <v>4</v>
       </c>
       <c r="B7" s="38">
-        <v>-0.17855825511226522</v>
+        <v>-0.13993747861363737</v>
       </c>
       <c r="C7" s="39">
-        <v>-0.35685101244146372</v>
+        <v>-0.27945448217603419</v>
       </c>
       <c r="D7" s="40">
         <v>1</v>
       </c>
       <c r="E7" s="41">
-        <v>0.25164832694089517</v>
+        <v>0.40155912864193949</v>
       </c>
       <c r="F7" s="42">
-        <v>0.46119388743585715</v>
+        <v>0.42912592330888261</v>
       </c>
       <c r="G7" s="43">
-        <v>0.30259070532716881</v>
+        <v>0.32019271326411253</v>
       </c>
       <c r="H7" s="44">
-        <v>-0.23369463866829404</v>
+        <v>0.21634283999811413</v>
       </c>
       <c r="I7" s="45">
-        <v>0.29338269259758537</v>
+        <v>0.11978361869829954</v>
       </c>
       <c r="J7" s="46">
-        <v>0.039728135770174193</v>
+        <v>0.04125258886298367</v>
       </c>
       <c r="K7" s="47">
-        <v>0.013196374556250948</v>
+        <v>0.0047140175651203941</v>
       </c>
       <c r="L7" s="48">
-        <v>0.21561891317541318</v>
+        <v>0.19410553124791485</v>
       </c>
     </row>
     <row r="8">
@@ -2429,37 +2429,37 @@
         <v>5</v>
       </c>
       <c r="B8" s="50">
-        <v>-0.13252929003989472</v>
+        <v>-0.072168942664718683</v>
       </c>
       <c r="C8" s="51">
-        <v>0.45723953115542315</v>
+        <v>0.3912405587965328</v>
       </c>
       <c r="D8" s="52">
-        <v>0.25164832694089517</v>
+        <v>0.40155912864193949</v>
       </c>
       <c r="E8" s="53">
         <v>1</v>
       </c>
       <c r="F8" s="54">
-        <v>0.036798517321935661</v>
+        <v>0.090803967982346856</v>
       </c>
       <c r="G8" s="55">
-        <v>0.27919005708008154</v>
+        <v>0.21811661040379263</v>
       </c>
       <c r="H8" s="56">
-        <v>0.56701095279980895</v>
+        <v>0.77340136336461285</v>
       </c>
       <c r="I8" s="57">
-        <v>0.62221565995712869</v>
+        <v>0.16091665801755389</v>
       </c>
       <c r="J8" s="58">
-        <v>0.087488741986652921</v>
+        <v>0.058432163892396222</v>
       </c>
       <c r="K8" s="59">
-        <v>-0.00013492808286029404</v>
+        <v>-0.014682406063411898</v>
       </c>
       <c r="L8" s="60">
-        <v>0.14964101469214922</v>
+        <v>0.12465952863273519</v>
       </c>
     </row>
     <row r="9">
@@ -2467,37 +2467,37 @@
         <v>6</v>
       </c>
       <c r="B9" s="62">
-        <v>-0.16158769856153238</v>
+        <v>-0.16020229891420215</v>
       </c>
       <c r="C9" s="63">
-        <v>-0.19866141481895314</v>
+        <v>-0.16779261703691015</v>
       </c>
       <c r="D9" s="64">
-        <v>0.46119388743585715</v>
+        <v>0.42912592330888261</v>
       </c>
       <c r="E9" s="65">
-        <v>0.036798517321935661</v>
+        <v>0.090803967982346856</v>
       </c>
       <c r="F9" s="66">
         <v>1</v>
       </c>
       <c r="G9" s="67">
-        <v>0.18686928409716475</v>
+        <v>0.12749728338120617</v>
       </c>
       <c r="H9" s="68">
-        <v>-0.60644440174382652</v>
+        <v>-0.2031264335750527</v>
       </c>
       <c r="I9" s="69">
-        <v>0.48728889194020614</v>
+        <v>0.34106670595667427</v>
       </c>
       <c r="J9" s="70">
-        <v>-0.047302388798186774</v>
+        <v>-0.060208231661128375</v>
       </c>
       <c r="K9" s="71">
-        <v>0.08143446124046215</v>
+        <v>0.07116969700858386</v>
       </c>
       <c r="L9" s="72">
-        <v>0.27365180282301732</v>
+        <v>0.25541188454012304</v>
       </c>
     </row>
     <row r="10">
@@ -2505,37 +2505,37 @@
         <v>7</v>
       </c>
       <c r="B10" s="74">
-        <v>-0.078605187138131694</v>
+        <v>-0.036455441011521955</v>
       </c>
       <c r="C10" s="75">
-        <v>-0.11068638947112709</v>
+        <v>-0.082947729960389002</v>
       </c>
       <c r="D10" s="76">
-        <v>0.30259070532716881</v>
+        <v>0.32019271326411253</v>
       </c>
       <c r="E10" s="77">
-        <v>0.27919005708008154</v>
+        <v>0.21811661040379263</v>
       </c>
       <c r="F10" s="78">
-        <v>0.18686928409716475</v>
+        <v>0.12749728338120617</v>
       </c>
       <c r="G10" s="79">
         <v>1</v>
       </c>
       <c r="H10" s="80">
-        <v>0.1770481427782592</v>
+        <v>0.18376831842116864</v>
       </c>
       <c r="I10" s="81">
-        <v>0.53177835681715946</v>
+        <v>0.41526573417468066</v>
       </c>
       <c r="J10" s="82">
-        <v>0.065025076008316932</v>
+        <v>0.080660175944025317</v>
       </c>
       <c r="K10" s="83">
-        <v>-0.0081701370092878908</v>
+        <v>-0.008810273659217778</v>
       </c>
       <c r="L10" s="84">
-        <v>0.11214024531845068</v>
+        <v>0.07947413633115552</v>
       </c>
     </row>
     <row r="11">
@@ -2543,37 +2543,37 @@
         <v>8</v>
       </c>
       <c r="B11" s="86">
-        <v>0.0039272163451361287</v>
+        <v>0.051208472342005616</v>
       </c>
       <c r="C11" s="87">
-        <v>0.35783377533033073</v>
+        <v>0.25181928605750192</v>
       </c>
       <c r="D11" s="88">
-        <v>-0.23369463866829404</v>
+        <v>0.21634283999811413</v>
       </c>
       <c r="E11" s="89">
-        <v>0.56701095279980895</v>
+        <v>0.77340136336461285</v>
       </c>
       <c r="F11" s="90">
-        <v>-0.60644440174382652</v>
+        <v>-0.2031264335750527</v>
       </c>
       <c r="G11" s="91">
-        <v>0.1770481427782592</v>
+        <v>0.18376831842116864</v>
       </c>
       <c r="H11" s="92">
         <v>1</v>
       </c>
       <c r="I11" s="93">
-        <v>0.16966854180303423</v>
+        <v>-0.22185946453849115</v>
       </c>
       <c r="J11" s="94">
-        <v>0.076394131005855959</v>
+        <v>0.041866580406255079</v>
       </c>
       <c r="K11" s="95">
-        <v>-0.06377435855605787</v>
+        <v>-0.04575927761463635</v>
       </c>
       <c r="L11" s="96">
-        <v>-0.073799580871541842</v>
+        <v>-0.014253467880990835</v>
       </c>
     </row>
     <row r="12">
@@ -2581,37 +2581,37 @@
         <v>9</v>
       </c>
       <c r="B12" s="98">
-        <v>-0.18790273986482514</v>
+        <v>-0.16107412495124424</v>
       </c>
       <c r="C12" s="99">
-        <v>0.18904785927448819</v>
+        <v>0.13795657281457507</v>
       </c>
       <c r="D12" s="100">
-        <v>0.29338269259758537</v>
+        <v>0.11978361869829954</v>
       </c>
       <c r="E12" s="101">
-        <v>0.62221565995712869</v>
+        <v>0.16091665801755389</v>
       </c>
       <c r="F12" s="102">
-        <v>0.48728889194020614</v>
+        <v>0.34106670595667427</v>
       </c>
       <c r="G12" s="103">
-        <v>0.53177835681715946</v>
+        <v>0.41526573417468066</v>
       </c>
       <c r="H12" s="104">
-        <v>0.16966854180303423</v>
+        <v>-0.22185946453849115</v>
       </c>
       <c r="I12" s="105">
         <v>1</v>
       </c>
       <c r="J12" s="106">
-        <v>0.065801818958581504</v>
+        <v>0.036733425298632667</v>
       </c>
       <c r="K12" s="107">
-        <v>0.039113137628966475</v>
+        <v>0.046601461405648886</v>
       </c>
       <c r="L12" s="108">
-        <v>0.24781664895007607</v>
+        <v>0.21262233168341874</v>
       </c>
     </row>
     <row r="13">
@@ -2619,37 +2619,37 @@
         <v>10</v>
       </c>
       <c r="B13" s="110">
-        <v>-0.086944371736145623</v>
+        <v>-0.074643708637271544</v>
       </c>
       <c r="C13" s="111">
-        <v>0.0082009235447547887</v>
+        <v>0.0034549274764648146</v>
       </c>
       <c r="D13" s="112">
-        <v>0.039728135770174193</v>
+        <v>0.04125258886298367</v>
       </c>
       <c r="E13" s="113">
-        <v>0.087488741986652921</v>
+        <v>0.058432163892396222</v>
       </c>
       <c r="F13" s="114">
-        <v>-0.047302388798186774</v>
+        <v>-0.060208231661128375</v>
       </c>
       <c r="G13" s="115">
-        <v>0.065025076008316932</v>
+        <v>0.080660175944025317</v>
       </c>
       <c r="H13" s="116">
-        <v>0.076394131005855959</v>
+        <v>0.041866580406255079</v>
       </c>
       <c r="I13" s="117">
-        <v>0.065801818958581504</v>
+        <v>0.036733425298632667</v>
       </c>
       <c r="J13" s="118">
         <v>1</v>
       </c>
       <c r="K13" s="119">
-        <v>-0.054931692707897301</v>
+        <v>-0.048841031051538378</v>
       </c>
       <c r="L13" s="120">
-        <v>-0.026839902465387953</v>
+        <v>-0.045254509277849436</v>
       </c>
     </row>
     <row r="14">
@@ -2657,37 +2657,37 @@
         <v>11</v>
       </c>
       <c r="B14" s="122">
-        <v>-0.053100175798924773</v>
+        <v>-0.053667623229320345</v>
       </c>
       <c r="C14" s="123">
-        <v>-0.0032735505005431517</v>
+        <v>-0.0051518167771299923</v>
       </c>
       <c r="D14" s="124">
-        <v>0.013196374556250948</v>
+        <v>0.0047140175651203941</v>
       </c>
       <c r="E14" s="125">
-        <v>-0.00013492808286029404</v>
+        <v>-0.014682406063411898</v>
       </c>
       <c r="F14" s="126">
-        <v>0.08143446124046215</v>
+        <v>0.07116969700858386</v>
       </c>
       <c r="G14" s="127">
-        <v>-0.0081701370092878908</v>
+        <v>-0.008810273659217778</v>
       </c>
       <c r="H14" s="128">
-        <v>-0.06377435855605787</v>
+        <v>-0.04575927761463635</v>
       </c>
       <c r="I14" s="129">
-        <v>0.039113137628966475</v>
+        <v>0.046601461405648886</v>
       </c>
       <c r="J14" s="130">
-        <v>-0.054931692707897301</v>
+        <v>-0.048841031051538378</v>
       </c>
       <c r="K14" s="131">
         <v>1</v>
       </c>
       <c r="L14" s="132">
-        <v>0.033268462495427857</v>
+        <v>0.029825345894238905</v>
       </c>
     </row>
     <row r="15">
@@ -2695,34 +2695,34 @@
         <v>12</v>
       </c>
       <c r="B15" s="134">
-        <v>-0.31364711226513603</v>
+        <v>-0.30695290477763448</v>
       </c>
       <c r="C15" s="135">
-        <v>-0.038354854119573539</v>
+        <v>-0.037623278440063204</v>
       </c>
       <c r="D15" s="136">
-        <v>0.21561891317541318</v>
+        <v>0.19410553124791485</v>
       </c>
       <c r="E15" s="137">
-        <v>0.14964101469214922</v>
+        <v>0.12465952863273519</v>
       </c>
       <c r="F15" s="138">
-        <v>0.27365180282301732</v>
+        <v>0.25541188454012304</v>
       </c>
       <c r="G15" s="139">
-        <v>0.11214024531845068</v>
+        <v>0.07947413633115552</v>
       </c>
       <c r="H15" s="140">
-        <v>-0.073799580871541842</v>
+        <v>-0.014253467880990835</v>
       </c>
       <c r="I15" s="141">
-        <v>0.24781664895007607</v>
+        <v>0.21262233168341874</v>
       </c>
       <c r="J15" s="142">
-        <v>-0.026839902465387953</v>
+        <v>-0.045254509277849436</v>
       </c>
       <c r="K15" s="143">
-        <v>0.033268462495427857</v>
+        <v>0.029825345894238905</v>
       </c>
       <c r="L15" s="144">
         <v>1</v>

</xml_diff>

<commit_message>
Restore fiscal balance control and refresh final FE-DK results
</commit_message>
<xml_diff>
--- a/src/econometrics/wp07_reestimation/Final_spec_correlation_matrix.xlsx
+++ b/src/econometrics/wp07_reestimation/Final_spec_correlation_matrix.xlsx
@@ -2318,34 +2318,34 @@
         <v>1</v>
       </c>
       <c r="C5" s="15">
-        <v>0.033988950952882471</v>
+        <v>0.033988950952882409</v>
       </c>
       <c r="D5" s="16">
         <v>-0.13993747861363737</v>
       </c>
       <c r="E5" s="17">
-        <v>-0.072168942664718683</v>
+        <v>-0.072168942664718641</v>
       </c>
       <c r="F5" s="18">
-        <v>-0.16020229891420215</v>
+        <v>-0.16020229891420212</v>
       </c>
       <c r="G5" s="19">
-        <v>-0.036455441011521955</v>
+        <v>-0.036455441011521934</v>
       </c>
       <c r="H5" s="20">
-        <v>0.051208472342005616</v>
+        <v>0.015585289228654079</v>
       </c>
       <c r="I5" s="21">
-        <v>-0.16107412495124424</v>
+        <v>-0.050588171973576256</v>
       </c>
       <c r="J5" s="22">
-        <v>-0.074643708637271544</v>
+        <v>-0.074643708637271489</v>
       </c>
       <c r="K5" s="23">
-        <v>-0.053667623229320345</v>
+        <v>-0.053667623229320359</v>
       </c>
       <c r="L5" s="24">
-        <v>-0.30695290477763448</v>
+        <v>-0.30695290477763454</v>
       </c>
     </row>
     <row r="6">
@@ -2353,7 +2353,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="26">
-        <v>0.033988950952882471</v>
+        <v>0.033988950952882409</v>
       </c>
       <c r="C6" s="27">
         <v>1</v>
@@ -2371,19 +2371,19 @@
         <v>-0.082947729960389002</v>
       </c>
       <c r="H6" s="32">
-        <v>0.25181928605750192</v>
+        <v>0.094696905124828035</v>
       </c>
       <c r="I6" s="33">
-        <v>0.13795657281457507</v>
+        <v>0.265462676630428</v>
       </c>
       <c r="J6" s="34">
-        <v>0.0034549274764648146</v>
+        <v>0.0034549274764648021</v>
       </c>
       <c r="K6" s="35">
-        <v>-0.0051518167771299923</v>
+        <v>-0.0051518167771299949</v>
       </c>
       <c r="L6" s="36">
-        <v>-0.037623278440063204</v>
+        <v>-0.03762327844006317</v>
       </c>
     </row>
     <row r="7">
@@ -2409,19 +2409,19 @@
         <v>0.32019271326411253</v>
       </c>
       <c r="H7" s="44">
-        <v>0.21634283999811413</v>
+        <v>-0.26351571306656679</v>
       </c>
       <c r="I7" s="45">
-        <v>0.11978361869829954</v>
+        <v>-0.082767954902241481</v>
       </c>
       <c r="J7" s="46">
-        <v>0.04125258886298367</v>
+        <v>0.041252588862983733</v>
       </c>
       <c r="K7" s="47">
-        <v>0.0047140175651203941</v>
+        <v>0.0047140175651203889</v>
       </c>
       <c r="L7" s="48">
-        <v>0.19410553124791485</v>
+        <v>0.19410553124791494</v>
       </c>
     </row>
     <row r="8">
@@ -2429,7 +2429,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="50">
-        <v>-0.072168942664718683</v>
+        <v>-0.072168942664718641</v>
       </c>
       <c r="C8" s="51">
         <v>0.3912405587965328</v>
@@ -2447,19 +2447,19 @@
         <v>0.21811661040379263</v>
       </c>
       <c r="H8" s="56">
-        <v>0.77340136336461285</v>
+        <v>-0.3829552461889858</v>
       </c>
       <c r="I8" s="57">
-        <v>0.16091665801755389</v>
+        <v>0.1186639165704597</v>
       </c>
       <c r="J8" s="58">
-        <v>0.058432163892396222</v>
+        <v>0.058432163892396208</v>
       </c>
       <c r="K8" s="59">
-        <v>-0.014682406063411898</v>
+        <v>-0.014682406063411899</v>
       </c>
       <c r="L8" s="60">
-        <v>0.12465952863273519</v>
+        <v>0.12465952863273509</v>
       </c>
     </row>
     <row r="9">
@@ -2467,7 +2467,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="62">
-        <v>-0.16020229891420215</v>
+        <v>-0.16020229891420212</v>
       </c>
       <c r="C9" s="63">
         <v>-0.16779261703691015</v>
@@ -2485,19 +2485,19 @@
         <v>0.12749728338120617</v>
       </c>
       <c r="H9" s="68">
-        <v>-0.2031264335750527</v>
+        <v>0.11369537029380532</v>
       </c>
       <c r="I9" s="69">
-        <v>0.34106670595667427</v>
+        <v>-0.089921555195720954</v>
       </c>
       <c r="J9" s="70">
-        <v>-0.060208231661128375</v>
+        <v>-0.060208231661128438</v>
       </c>
       <c r="K9" s="71">
-        <v>0.07116969700858386</v>
+        <v>0.071169697008583888</v>
       </c>
       <c r="L9" s="72">
-        <v>0.25541188454012304</v>
+        <v>0.25541188454012309</v>
       </c>
     </row>
     <row r="10">
@@ -2505,7 +2505,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="74">
-        <v>-0.036455441011521955</v>
+        <v>-0.036455441011521934</v>
       </c>
       <c r="C10" s="75">
         <v>-0.082947729960389002</v>
@@ -2523,19 +2523,19 @@
         <v>1</v>
       </c>
       <c r="H10" s="80">
-        <v>0.18376831842116864</v>
+        <v>0.3611426677562769</v>
       </c>
       <c r="I10" s="81">
-        <v>0.41526573417468066</v>
+        <v>0.23323545582631811</v>
       </c>
       <c r="J10" s="82">
-        <v>0.080660175944025317</v>
+        <v>0.080660175944025303</v>
       </c>
       <c r="K10" s="83">
-        <v>-0.008810273659217778</v>
+        <v>-0.0088102736592178005</v>
       </c>
       <c r="L10" s="84">
-        <v>0.07947413633115552</v>
+        <v>0.079474136331155562</v>
       </c>
     </row>
     <row r="11">
@@ -2543,37 +2543,37 @@
         <v>8</v>
       </c>
       <c r="B11" s="86">
-        <v>0.051208472342005616</v>
+        <v>0.015585289228654079</v>
       </c>
       <c r="C11" s="87">
-        <v>0.25181928605750192</v>
+        <v>0.094696905124828035</v>
       </c>
       <c r="D11" s="88">
-        <v>0.21634283999811413</v>
+        <v>-0.26351571306656679</v>
       </c>
       <c r="E11" s="89">
-        <v>0.77340136336461285</v>
+        <v>-0.3829552461889858</v>
       </c>
       <c r="F11" s="90">
-        <v>-0.2031264335750527</v>
+        <v>0.11369537029380532</v>
       </c>
       <c r="G11" s="91">
-        <v>0.18376831842116864</v>
+        <v>0.3611426677562769</v>
       </c>
       <c r="H11" s="92">
         <v>1</v>
       </c>
       <c r="I11" s="93">
-        <v>-0.22185946453849115</v>
+        <v>0.22941400141223697</v>
       </c>
       <c r="J11" s="94">
-        <v>0.041866580406255079</v>
+        <v>-0.0031787591336458689</v>
       </c>
       <c r="K11" s="95">
-        <v>-0.04575927761463635</v>
+        <v>0.054828429527539836</v>
       </c>
       <c r="L11" s="96">
-        <v>-0.014253467880990835</v>
+        <v>-0.021205540647933948</v>
       </c>
     </row>
     <row r="12">
@@ -2581,37 +2581,37 @@
         <v>9</v>
       </c>
       <c r="B12" s="98">
-        <v>-0.16107412495124424</v>
+        <v>-0.050588171973576256</v>
       </c>
       <c r="C12" s="99">
-        <v>0.13795657281457507</v>
+        <v>0.265462676630428</v>
       </c>
       <c r="D12" s="100">
-        <v>0.11978361869829954</v>
+        <v>-0.082767954902241481</v>
       </c>
       <c r="E12" s="101">
-        <v>0.16091665801755389</v>
+        <v>0.1186639165704597</v>
       </c>
       <c r="F12" s="102">
-        <v>0.34106670595667427</v>
+        <v>-0.089921555195720954</v>
       </c>
       <c r="G12" s="103">
-        <v>0.41526573417468066</v>
+        <v>0.23323545582631811</v>
       </c>
       <c r="H12" s="104">
-        <v>-0.22185946453849115</v>
+        <v>0.22941400141223697</v>
       </c>
       <c r="I12" s="105">
         <v>1</v>
       </c>
       <c r="J12" s="106">
-        <v>0.036733425298632667</v>
+        <v>0.0052272994250406263</v>
       </c>
       <c r="K12" s="107">
-        <v>0.046601461405648886</v>
+        <v>0.02523650491384738</v>
       </c>
       <c r="L12" s="108">
-        <v>0.21262233168341874</v>
+        <v>0.14854284112811147</v>
       </c>
     </row>
     <row r="13">
@@ -2619,37 +2619,37 @@
         <v>10</v>
       </c>
       <c r="B13" s="110">
-        <v>-0.074643708637271544</v>
+        <v>-0.074643708637271489</v>
       </c>
       <c r="C13" s="111">
-        <v>0.0034549274764648146</v>
+        <v>0.0034549274764648021</v>
       </c>
       <c r="D13" s="112">
-        <v>0.04125258886298367</v>
+        <v>0.041252588862983733</v>
       </c>
       <c r="E13" s="113">
-        <v>0.058432163892396222</v>
+        <v>0.058432163892396208</v>
       </c>
       <c r="F13" s="114">
-        <v>-0.060208231661128375</v>
+        <v>-0.060208231661128438</v>
       </c>
       <c r="G13" s="115">
-        <v>0.080660175944025317</v>
+        <v>0.080660175944025303</v>
       </c>
       <c r="H13" s="116">
-        <v>0.041866580406255079</v>
+        <v>-0.0031787591336458689</v>
       </c>
       <c r="I13" s="117">
-        <v>0.036733425298632667</v>
+        <v>0.0052272994250406263</v>
       </c>
       <c r="J13" s="118">
         <v>1</v>
       </c>
       <c r="K13" s="119">
-        <v>-0.048841031051538378</v>
+        <v>-0.048841031051538392</v>
       </c>
       <c r="L13" s="120">
-        <v>-0.045254509277849436</v>
+        <v>-0.045254509277849443</v>
       </c>
     </row>
     <row r="14">
@@ -2657,37 +2657,37 @@
         <v>11</v>
       </c>
       <c r="B14" s="122">
-        <v>-0.053667623229320345</v>
+        <v>-0.053667623229320359</v>
       </c>
       <c r="C14" s="123">
-        <v>-0.0051518167771299923</v>
+        <v>-0.0051518167771299949</v>
       </c>
       <c r="D14" s="124">
-        <v>0.0047140175651203941</v>
+        <v>0.0047140175651203889</v>
       </c>
       <c r="E14" s="125">
-        <v>-0.014682406063411898</v>
+        <v>-0.014682406063411899</v>
       </c>
       <c r="F14" s="126">
-        <v>0.07116969700858386</v>
+        <v>0.071169697008583888</v>
       </c>
       <c r="G14" s="127">
-        <v>-0.008810273659217778</v>
+        <v>-0.0088102736592178005</v>
       </c>
       <c r="H14" s="128">
-        <v>-0.04575927761463635</v>
+        <v>0.054828429527539836</v>
       </c>
       <c r="I14" s="129">
-        <v>0.046601461405648886</v>
+        <v>0.02523650491384738</v>
       </c>
       <c r="J14" s="130">
-        <v>-0.048841031051538378</v>
+        <v>-0.048841031051538392</v>
       </c>
       <c r="K14" s="131">
         <v>1</v>
       </c>
       <c r="L14" s="132">
-        <v>0.029825345894238905</v>
+        <v>0.029825345894238894</v>
       </c>
     </row>
     <row r="15">
@@ -2695,34 +2695,34 @@
         <v>12</v>
       </c>
       <c r="B15" s="134">
-        <v>-0.30695290477763448</v>
+        <v>-0.30695290477763454</v>
       </c>
       <c r="C15" s="135">
-        <v>-0.037623278440063204</v>
+        <v>-0.03762327844006317</v>
       </c>
       <c r="D15" s="136">
-        <v>0.19410553124791485</v>
+        <v>0.19410553124791494</v>
       </c>
       <c r="E15" s="137">
-        <v>0.12465952863273519</v>
+        <v>0.12465952863273509</v>
       </c>
       <c r="F15" s="138">
-        <v>0.25541188454012304</v>
+        <v>0.25541188454012309</v>
       </c>
       <c r="G15" s="139">
-        <v>0.07947413633115552</v>
+        <v>0.079474136331155562</v>
       </c>
       <c r="H15" s="140">
-        <v>-0.014253467880990835</v>
+        <v>-0.021205540647933948</v>
       </c>
       <c r="I15" s="141">
-        <v>0.21262233168341874</v>
+        <v>0.14854284112811147</v>
       </c>
       <c r="J15" s="142">
-        <v>-0.045254509277849436</v>
+        <v>-0.045254509277849443</v>
       </c>
       <c r="K15" s="143">
-        <v>0.029825345894238905</v>
+        <v>0.029825345894238894</v>
       </c>
       <c r="L15" s="144">
         <v>1</v>

</xml_diff>